<commit_message>
feat: accumulate weekly sales and item prices
</commit_message>
<xml_diff>
--- a/assets/weekly_inventory_template.xlsx
+++ b/assets/weekly_inventory_template.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="재고현황" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="실재고 전산비교" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="재고데이터" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="재고데이터-리큐엠" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="재고데이터-위킵" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="재고데이터-이모아이" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="RAWDATA_이카운트" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DAILY" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="단가 " sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고현황" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실재고 전산비교" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고데이터" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고데이터-리큐엠" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고데이터-위킵" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고데이터-이모아이" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAWDATA_이카운트" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DAILY" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="단가 " sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId10"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
   </externalReferences>
   <definedNames>
     <definedName name="arial">#REF!</definedName>
@@ -33,6 +33,7 @@
     <definedName name="중복확인" localSheetId="1">#REF!+#REF!</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'재고데이터'!$2:$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'재고데이터-위킵'!$C$1:$C$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'RAWDATA_이카운트'!$A$2:$P$138710</definedName>
   </definedNames>
   <calcPr calcId="181029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1750,7 +1751,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1222">
+  <cellXfs count="1231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5408,6 +5409,33 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="22" fillId="0" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="10" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="45" fillId="10" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="76" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="77" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="83" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -5475,8 +5503,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="KT서부"/>
       <sheetName val="견적서"/>
@@ -27271,46 +27299,143 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor theme="1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="16.5"/>
+  <cols>
+    <col width="7.125" bestFit="1" customWidth="1" style="6" min="1" max="3"/>
+    <col width="8.625" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="8.625" customWidth="1" style="6" min="5" max="5"/>
+    <col width="0.125" customWidth="1" style="6" min="6" max="6"/>
+    <col width="10.875" customWidth="1" style="6" min="7" max="7"/>
+    <col width="12.125" customWidth="1" style="6" min="8" max="8"/>
+    <col width="15.5" customWidth="1" style="6" min="9" max="9"/>
+    <col width="44.5" customWidth="1" style="6" min="10" max="10"/>
+    <col width="21.625" bestFit="1" customWidth="1" style="6" min="11" max="11"/>
+    <col width="70.625" bestFit="1" customWidth="1" style="6" min="12" max="12"/>
+    <col width="8.625" bestFit="1" customWidth="1" style="6" min="13" max="13"/>
+    <col width="12" bestFit="1" customWidth="1" style="6" min="14" max="14"/>
+    <col width="10.375" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col width="9.375" bestFit="1" customWidth="1" style="6" min="16" max="16"/>
+    <col width="9" customWidth="1" style="5" min="17" max="72"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>기준일시</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>창고코드</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>창고명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>품목코드</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>품목명</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>현재고</t>
-        </is>
-      </c>
-    </row>
+      <c r="A1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="B1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,4,FALSE)</f>
+        <v/>
+      </c>
+      <c r="C1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,6,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,7,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F1" s="8">
+        <f>VLOOKUP($H1,DAILY!$C:$K,9,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>월</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>요일</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>주차</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>구간</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일별	</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">거래처코드	</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">거래처	</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">품목명[규격]코드	</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">품목명[규격]	</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">수량	</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공급가액	</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">부가세	</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합계	</t>
+        </is>
+      </c>
+    </row>
+    <row r="28315" ht="15.75" customHeight="1" s="744"/>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A2:P138710"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -27338,20 +27463,2043 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor theme="1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H336"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.5"/>
+  <cols>
+    <col collapsed="1" width="21.125" customWidth="1" style="744" min="1" max="1"/>
+    <col collapsed="1" width="34.75" customWidth="1" style="744" min="2" max="2"/>
+    <col collapsed="1" width="18.125" customWidth="1" style="744" min="3" max="3"/>
+    <col width="18.125" customWidth="1" style="820" min="4" max="4"/>
+    <col width="9" customWidth="1" style="717" min="5" max="16384"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>현재 단계에서는 단가 데이터 제외</t>
-        </is>
-      </c>
+      <c r="A1" s="554" t="inlineStr">
+        <is>
+          <t>회사명 : 주식회사 리큐엠 / 2026/07/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="556" t="inlineStr">
+        <is>
+          <t>품목코드</t>
+        </is>
+      </c>
+      <c r="B2" s="556" t="inlineStr">
+        <is>
+          <t>품목명[규격]</t>
+        </is>
+      </c>
+      <c r="C2" s="556" t="inlineStr">
+        <is>
+          <t>재고단가</t>
+        </is>
+      </c>
+      <c r="D2" s="1222" t="inlineStr">
+        <is>
+          <t>재고단가(+v)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="555" t="n"/>
+      <c r="B3" s="555" t="n"/>
+      <c r="C3" s="1223" t="n"/>
+      <c r="D3" s="1224" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="555" t="n"/>
+      <c r="B4" s="555" t="n"/>
+      <c r="C4" s="1223" t="n"/>
+      <c r="D4" s="1224" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="555" t="n"/>
+      <c r="B5" s="555" t="n"/>
+      <c r="C5" s="1223" t="n"/>
+      <c r="D5" s="1224" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="555" t="n"/>
+      <c r="B6" s="555" t="n"/>
+      <c r="C6" s="1223" t="n"/>
+      <c r="D6" s="1224" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="555" t="n"/>
+      <c r="B7" s="555" t="n"/>
+      <c r="C7" s="1223" t="n"/>
+      <c r="D7" s="1224" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="555" t="n"/>
+      <c r="B8" s="555" t="n"/>
+      <c r="C8" s="1223" t="n"/>
+      <c r="D8" s="1224" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="555" t="n"/>
+      <c r="B9" s="555" t="n"/>
+      <c r="C9" s="1223" t="n"/>
+      <c r="D9" s="1224" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="555" t="n"/>
+      <c r="B10" s="555" t="n"/>
+      <c r="C10" s="1223" t="n"/>
+      <c r="D10" s="1224" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="555" t="n"/>
+      <c r="B11" s="555" t="n"/>
+      <c r="C11" s="1223" t="n"/>
+      <c r="D11" s="1225" t="n"/>
+      <c r="H11" s="1226" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="555" t="n"/>
+      <c r="B12" s="555" t="n"/>
+      <c r="C12" s="1223" t="n"/>
+      <c r="D12" s="1225" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="555" t="n"/>
+      <c r="B13" s="555" t="n"/>
+      <c r="C13" s="1223" t="n"/>
+      <c r="D13" s="1225" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="555" t="n"/>
+      <c r="B14" s="555" t="n"/>
+      <c r="C14" s="1223" t="n"/>
+      <c r="D14" s="1225" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="555" t="n"/>
+      <c r="B15" s="555" t="n"/>
+      <c r="C15" s="1223" t="n"/>
+      <c r="D15" s="1225" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="555" t="n"/>
+      <c r="B16" s="555" t="n"/>
+      <c r="C16" s="1223" t="n"/>
+      <c r="D16" s="1225" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="555" t="n"/>
+      <c r="B17" s="555" t="n"/>
+      <c r="C17" s="1223" t="n"/>
+      <c r="D17" s="1225" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="555" t="n"/>
+      <c r="B18" s="555" t="n"/>
+      <c r="C18" s="1223" t="n"/>
+      <c r="D18" s="1225" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="555" t="n"/>
+      <c r="B19" s="555" t="n"/>
+      <c r="C19" s="1223" t="n"/>
+      <c r="D19" s="1225" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="555" t="n"/>
+      <c r="B20" s="555" t="n"/>
+      <c r="C20" s="1223" t="n"/>
+      <c r="D20" s="1225" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="555" t="n"/>
+      <c r="B21" s="555" t="n"/>
+      <c r="C21" s="1223" t="n"/>
+      <c r="D21" s="1225" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="555" t="n"/>
+      <c r="B22" s="555" t="n"/>
+      <c r="C22" s="1223" t="n"/>
+      <c r="D22" s="1225" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="555" t="n"/>
+      <c r="B23" s="555" t="n"/>
+      <c r="C23" s="1223" t="n"/>
+      <c r="D23" s="1225" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="555" t="n"/>
+      <c r="B24" s="555" t="n"/>
+      <c r="C24" s="1223" t="n"/>
+      <c r="D24" s="1225" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="555" t="n"/>
+      <c r="B25" s="555" t="n"/>
+      <c r="C25" s="1223" t="n"/>
+      <c r="D25" s="1225" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="555" t="n"/>
+      <c r="B26" s="555" t="n"/>
+      <c r="C26" s="1223" t="n"/>
+      <c r="D26" s="1225" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="555" t="n"/>
+      <c r="B27" s="555" t="n"/>
+      <c r="C27" s="1223" t="n"/>
+      <c r="D27" s="1225" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="555" t="n"/>
+      <c r="B28" s="555" t="n"/>
+      <c r="C28" s="1223" t="n"/>
+      <c r="D28" s="1225" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="555" t="n"/>
+      <c r="B29" s="555" t="n"/>
+      <c r="C29" s="1223" t="n"/>
+      <c r="D29" s="1225" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="555" t="n"/>
+      <c r="B30" s="555" t="n"/>
+      <c r="C30" s="1223" t="n"/>
+      <c r="D30" s="1225" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="555" t="n"/>
+      <c r="B31" s="555" t="n"/>
+      <c r="C31" s="1223" t="n"/>
+      <c r="D31" s="1225" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="555" t="n"/>
+      <c r="B32" s="555" t="n"/>
+      <c r="C32" s="1223" t="n"/>
+      <c r="D32" s="1225" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="555" t="n"/>
+      <c r="B33" s="555" t="n"/>
+      <c r="C33" s="1223" t="n"/>
+      <c r="D33" s="1225" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="555" t="n"/>
+      <c r="B34" s="555" t="n"/>
+      <c r="C34" s="1223" t="n"/>
+      <c r="D34" s="1225" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="555" t="n"/>
+      <c r="B35" s="555" t="n"/>
+      <c r="C35" s="1223" t="n"/>
+      <c r="D35" s="1224" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="555" t="n"/>
+      <c r="B36" s="555" t="n"/>
+      <c r="C36" s="1223" t="n"/>
+      <c r="D36" s="1224" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="555" t="n"/>
+      <c r="B37" s="555" t="n"/>
+      <c r="C37" s="1223" t="n"/>
+      <c r="D37" s="1224" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="555" t="n"/>
+      <c r="B38" s="555" t="n"/>
+      <c r="C38" s="1223" t="n"/>
+      <c r="D38" s="1224" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="555" t="n"/>
+      <c r="B39" s="555" t="n"/>
+      <c r="C39" s="1223" t="n"/>
+      <c r="D39" s="1224" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="555" t="n"/>
+      <c r="B40" s="555" t="n"/>
+      <c r="C40" s="1223" t="n"/>
+      <c r="D40" s="1224" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="555" t="n"/>
+      <c r="B41" s="555" t="n"/>
+      <c r="C41" s="1223" t="n"/>
+      <c r="D41" s="1224" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="555" t="n"/>
+      <c r="B42" s="555" t="n"/>
+      <c r="C42" s="1223" t="n"/>
+      <c r="D42" s="1224" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="555" t="n"/>
+      <c r="B43" s="555" t="n"/>
+      <c r="C43" s="1223" t="n"/>
+      <c r="D43" s="1224" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="555" t="n"/>
+      <c r="B44" s="555" t="n"/>
+      <c r="C44" s="1223" t="n"/>
+      <c r="D44" s="1224" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="555" t="n"/>
+      <c r="B45" s="555" t="n"/>
+      <c r="C45" s="1223" t="n"/>
+      <c r="D45" s="1224" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="555" t="n"/>
+      <c r="B46" s="555" t="n"/>
+      <c r="C46" s="1223" t="n"/>
+      <c r="D46" s="1224" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="555" t="n"/>
+      <c r="B47" s="555" t="n"/>
+      <c r="C47" s="1223" t="n"/>
+      <c r="D47" s="1224" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="555" t="n"/>
+      <c r="B48" s="555" t="n"/>
+      <c r="C48" s="1223" t="n"/>
+      <c r="D48" s="1224" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="555" t="n"/>
+      <c r="B49" s="555" t="n"/>
+      <c r="C49" s="1223" t="n"/>
+      <c r="D49" s="1224" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="555" t="n"/>
+      <c r="B50" s="555" t="n"/>
+      <c r="C50" s="1223" t="n"/>
+      <c r="D50" s="1224" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="555" t="n"/>
+      <c r="B51" s="555" t="n"/>
+      <c r="C51" s="1223" t="n"/>
+      <c r="D51" s="1224" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="555" t="n"/>
+      <c r="B52" s="555" t="n"/>
+      <c r="C52" s="1223" t="n"/>
+      <c r="D52" s="1224" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="555" t="n"/>
+      <c r="B53" s="555" t="n"/>
+      <c r="C53" s="1223" t="n"/>
+      <c r="D53" s="1224" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="555" t="n"/>
+      <c r="B54" s="555" t="n"/>
+      <c r="C54" s="1223" t="n"/>
+      <c r="D54" s="1224" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="555" t="n"/>
+      <c r="B55" s="555" t="n"/>
+      <c r="C55" s="1223" t="n"/>
+      <c r="D55" s="1224" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="555" t="n"/>
+      <c r="B56" s="555" t="n"/>
+      <c r="C56" s="1223" t="n"/>
+      <c r="D56" s="1224" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="555" t="n"/>
+      <c r="B57" s="555" t="n"/>
+      <c r="C57" s="1223" t="n"/>
+      <c r="D57" s="1224" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="555" t="n"/>
+      <c r="B58" s="555" t="n"/>
+      <c r="C58" s="1223" t="n"/>
+      <c r="D58" s="1224" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="555" t="n"/>
+      <c r="B59" s="555" t="n"/>
+      <c r="C59" s="1223" t="n"/>
+      <c r="D59" s="1224" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="555" t="n"/>
+      <c r="B60" s="555" t="n"/>
+      <c r="C60" s="1223" t="n"/>
+      <c r="D60" s="1224" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="555" t="n"/>
+      <c r="B61" s="555" t="n"/>
+      <c r="C61" s="1223" t="n"/>
+      <c r="D61" s="1224" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="555" t="n"/>
+      <c r="B62" s="555" t="n"/>
+      <c r="C62" s="1223" t="n"/>
+      <c r="D62" s="1224" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="555" t="n"/>
+      <c r="B63" s="555" t="n"/>
+      <c r="C63" s="1223" t="n"/>
+      <c r="D63" s="1224" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="555" t="n"/>
+      <c r="B64" s="555" t="n"/>
+      <c r="C64" s="1223" t="n"/>
+      <c r="D64" s="1224" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="555" t="n"/>
+      <c r="B65" s="555" t="n"/>
+      <c r="C65" s="1223" t="n"/>
+      <c r="D65" s="1224" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="555" t="n"/>
+      <c r="B66" s="555" t="n"/>
+      <c r="C66" s="1223" t="n"/>
+      <c r="D66" s="1224" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="555" t="n"/>
+      <c r="B67" s="555" t="n"/>
+      <c r="C67" s="1223" t="n"/>
+      <c r="D67" s="1224" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="555" t="n"/>
+      <c r="B68" s="555" t="n"/>
+      <c r="C68" s="1223" t="n"/>
+      <c r="D68" s="1224" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="555" t="n"/>
+      <c r="B69" s="555" t="n"/>
+      <c r="C69" s="1223" t="n"/>
+      <c r="D69" s="1224" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="555" t="n"/>
+      <c r="B70" s="555" t="n"/>
+      <c r="C70" s="1223" t="n"/>
+      <c r="D70" s="1224" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="555" t="n"/>
+      <c r="B71" s="555" t="n"/>
+      <c r="C71" s="1223" t="n"/>
+      <c r="D71" s="1224" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="555" t="n"/>
+      <c r="B72" s="555" t="n"/>
+      <c r="C72" s="1223" t="n"/>
+      <c r="D72" s="1224" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="555" t="n"/>
+      <c r="B73" s="555" t="n"/>
+      <c r="C73" s="1223" t="n"/>
+      <c r="D73" s="1224" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="555" t="n"/>
+      <c r="B74" s="555" t="n"/>
+      <c r="C74" s="1223" t="n"/>
+      <c r="D74" s="1224" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="555" t="n"/>
+      <c r="B75" s="555" t="n"/>
+      <c r="C75" s="1223" t="n"/>
+      <c r="D75" s="1224" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="555" t="n"/>
+      <c r="B76" s="555" t="n"/>
+      <c r="C76" s="1223" t="n"/>
+      <c r="D76" s="1224" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="555" t="n"/>
+      <c r="B77" s="555" t="n"/>
+      <c r="C77" s="1223" t="n"/>
+      <c r="D77" s="1224" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="555" t="n"/>
+      <c r="B78" s="555" t="n"/>
+      <c r="C78" s="1223" t="n"/>
+      <c r="D78" s="1224" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="555" t="n"/>
+      <c r="B79" s="555" t="n"/>
+      <c r="C79" s="1223" t="n"/>
+      <c r="D79" s="1224" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="555" t="n"/>
+      <c r="B80" s="555" t="n"/>
+      <c r="C80" s="1223" t="n"/>
+      <c r="D80" s="1224" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="555" t="n"/>
+      <c r="B81" s="555" t="n"/>
+      <c r="C81" s="1223" t="n"/>
+      <c r="D81" s="1224" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="555" t="n"/>
+      <c r="B82" s="555" t="n"/>
+      <c r="C82" s="1223" t="n"/>
+      <c r="D82" s="1224" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="555" t="n"/>
+      <c r="B83" s="555" t="n"/>
+      <c r="C83" s="1223" t="n"/>
+      <c r="D83" s="1224" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="555" t="n"/>
+      <c r="B84" s="555" t="n"/>
+      <c r="C84" s="1223" t="n"/>
+      <c r="D84" s="1224" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="555" t="n"/>
+      <c r="B85" s="555" t="n"/>
+      <c r="C85" s="1223" t="n"/>
+      <c r="D85" s="1224" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="555" t="n"/>
+      <c r="B86" s="555" t="n"/>
+      <c r="C86" s="1223" t="n"/>
+      <c r="D86" s="1224" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="555" t="n"/>
+      <c r="B87" s="555" t="n"/>
+      <c r="C87" s="1223" t="n"/>
+      <c r="D87" s="1224" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="555" t="n"/>
+      <c r="B88" s="555" t="n"/>
+      <c r="C88" s="1223" t="n"/>
+      <c r="D88" s="1224" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="555" t="n"/>
+      <c r="B89" s="555" t="n"/>
+      <c r="C89" s="1223" t="n"/>
+      <c r="D89" s="1224" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="555" t="n"/>
+      <c r="B90" s="555" t="n"/>
+      <c r="C90" s="1223" t="n"/>
+      <c r="D90" s="1224" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="555" t="n"/>
+      <c r="B91" s="555" t="n"/>
+      <c r="C91" s="1223" t="n"/>
+      <c r="D91" s="1224" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="555" t="n"/>
+      <c r="B92" s="555" t="n"/>
+      <c r="C92" s="1223" t="n"/>
+      <c r="D92" s="1224" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="555" t="n"/>
+      <c r="B93" s="555" t="n"/>
+      <c r="C93" s="1223" t="n"/>
+      <c r="D93" s="1224" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="555" t="n"/>
+      <c r="B94" s="555" t="n"/>
+      <c r="C94" s="1223" t="n"/>
+      <c r="D94" s="1224" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="555" t="n"/>
+      <c r="B95" s="555" t="n"/>
+      <c r="C95" s="1223" t="n"/>
+      <c r="D95" s="1224" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="555" t="n"/>
+      <c r="B96" s="555" t="n"/>
+      <c r="C96" s="1223" t="n"/>
+      <c r="D96" s="1224" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="555" t="n"/>
+      <c r="B97" s="555" t="n"/>
+      <c r="C97" s="1223" t="n"/>
+      <c r="D97" s="1224" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="555" t="n"/>
+      <c r="B98" s="555" t="n"/>
+      <c r="C98" s="1223" t="n"/>
+      <c r="D98" s="1224" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="555" t="n"/>
+      <c r="B99" s="555" t="n"/>
+      <c r="C99" s="1223" t="n"/>
+      <c r="D99" s="1224" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="555" t="n"/>
+      <c r="B100" s="555" t="n"/>
+      <c r="C100" s="1223" t="n"/>
+      <c r="D100" s="1224" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="555" t="n"/>
+      <c r="B101" s="555" t="n"/>
+      <c r="C101" s="1223" t="n"/>
+      <c r="D101" s="1224" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="555" t="n"/>
+      <c r="B102" s="555" t="n"/>
+      <c r="C102" s="1223" t="n"/>
+      <c r="D102" s="1224" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="555" t="n"/>
+      <c r="B103" s="555" t="n"/>
+      <c r="C103" s="1223" t="n"/>
+      <c r="D103" s="1227" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="555" t="n"/>
+      <c r="B104" s="555" t="n"/>
+      <c r="C104" s="1223" t="n"/>
+      <c r="D104" s="1228" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="555" t="n"/>
+      <c r="B105" s="555" t="n"/>
+      <c r="C105" s="1223" t="n"/>
+      <c r="D105" s="1228" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="555" t="n"/>
+      <c r="B106" s="555" t="n"/>
+      <c r="C106" s="1223" t="n"/>
+      <c r="D106" s="1228" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="555" t="n"/>
+      <c r="B107" s="555" t="n"/>
+      <c r="C107" s="1223" t="n"/>
+      <c r="D107" s="1228" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="555" t="n"/>
+      <c r="B108" s="555" t="n"/>
+      <c r="C108" s="1223" t="n"/>
+      <c r="D108" s="1228" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="555" t="n"/>
+      <c r="B109" s="555" t="n"/>
+      <c r="C109" s="1223" t="n"/>
+      <c r="D109" s="1228" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="555" t="n"/>
+      <c r="B110" s="555" t="n"/>
+      <c r="C110" s="1223" t="n"/>
+      <c r="D110" s="1228" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="555" t="n"/>
+      <c r="B111" s="555" t="n"/>
+      <c r="C111" s="1223" t="n"/>
+      <c r="D111" s="1228" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="555" t="n"/>
+      <c r="B112" s="555" t="n"/>
+      <c r="C112" s="1223" t="n"/>
+      <c r="D112" s="1228" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="555" t="n"/>
+      <c r="B113" s="555" t="n"/>
+      <c r="C113" s="1223" t="n"/>
+      <c r="D113" s="1228" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="555" t="n"/>
+      <c r="B114" s="555" t="n"/>
+      <c r="C114" s="1223" t="n"/>
+      <c r="D114" s="1228" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="555" t="n"/>
+      <c r="B115" s="555" t="n"/>
+      <c r="C115" s="1223" t="n"/>
+      <c r="D115" s="1228" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="555" t="n"/>
+      <c r="B116" s="555" t="n"/>
+      <c r="C116" s="1223" t="n"/>
+      <c r="D116" s="1228" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="555" t="n"/>
+      <c r="B117" s="555" t="n"/>
+      <c r="C117" s="1223" t="n"/>
+      <c r="D117" s="1228" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="555" t="n"/>
+      <c r="B118" s="555" t="n"/>
+      <c r="C118" s="1223" t="n"/>
+      <c r="D118" s="1228" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="555" t="n"/>
+      <c r="B119" s="555" t="n"/>
+      <c r="C119" s="1223" t="n"/>
+      <c r="D119" s="1228" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="555" t="n"/>
+      <c r="B120" s="555" t="n"/>
+      <c r="C120" s="1223" t="n"/>
+      <c r="D120" s="1228" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="555" t="n"/>
+      <c r="B121" s="555" t="n"/>
+      <c r="C121" s="1223" t="n"/>
+      <c r="D121" s="1228" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="555" t="n"/>
+      <c r="B122" s="555" t="n"/>
+      <c r="C122" s="1223" t="n"/>
+      <c r="D122" s="1228" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="555" t="n"/>
+      <c r="B123" s="555" t="n"/>
+      <c r="C123" s="1223" t="n"/>
+      <c r="D123" s="1228" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="555" t="n"/>
+      <c r="B124" s="555" t="n"/>
+      <c r="C124" s="1223" t="n"/>
+      <c r="D124" s="1228" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="555" t="n"/>
+      <c r="B125" s="555" t="n"/>
+      <c r="C125" s="1223" t="n"/>
+      <c r="D125" s="1228" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="555" t="n"/>
+      <c r="B126" s="555" t="n"/>
+      <c r="C126" s="1223" t="n"/>
+      <c r="D126" s="1228" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="555" t="n"/>
+      <c r="B127" s="555" t="n"/>
+      <c r="C127" s="1223" t="n"/>
+      <c r="D127" s="1228" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="555" t="n"/>
+      <c r="B128" s="555" t="n"/>
+      <c r="C128" s="1223" t="n"/>
+      <c r="D128" s="1228" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="555" t="n"/>
+      <c r="B129" s="555" t="n"/>
+      <c r="C129" s="1223" t="n"/>
+      <c r="D129" s="1228" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="555" t="n"/>
+      <c r="B130" s="555" t="n"/>
+      <c r="C130" s="1223" t="n"/>
+      <c r="D130" s="1228" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="555" t="n"/>
+      <c r="B131" s="555" t="n"/>
+      <c r="C131" s="1223" t="n"/>
+      <c r="D131" s="1228" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="555" t="n"/>
+      <c r="B132" s="555" t="n"/>
+      <c r="C132" s="1223" t="n"/>
+      <c r="D132" s="1228" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="555" t="n"/>
+      <c r="B133" s="555" t="n"/>
+      <c r="C133" s="1223" t="n"/>
+      <c r="D133" s="1228" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="555" t="n"/>
+      <c r="B134" s="555" t="n"/>
+      <c r="C134" s="1223" t="n"/>
+      <c r="D134" s="1228" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="555" t="n"/>
+      <c r="B135" s="555" t="n"/>
+      <c r="C135" s="1223" t="n"/>
+      <c r="D135" s="1228" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="555" t="n"/>
+      <c r="B136" s="555" t="n"/>
+      <c r="C136" s="1223" t="n"/>
+      <c r="D136" s="1228" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="555" t="n"/>
+      <c r="B137" s="555" t="n"/>
+      <c r="C137" s="1223" t="n"/>
+      <c r="D137" s="1228" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="555" t="n"/>
+      <c r="B138" s="555" t="n"/>
+      <c r="C138" s="1223" t="n"/>
+      <c r="D138" s="1228" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="555" t="n"/>
+      <c r="B139" s="555" t="n"/>
+      <c r="C139" s="1223" t="n"/>
+      <c r="D139" s="1228" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="555" t="n"/>
+      <c r="B140" s="555" t="n"/>
+      <c r="C140" s="1223" t="n"/>
+      <c r="D140" s="1228" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="555" t="n"/>
+      <c r="B141" s="555" t="n"/>
+      <c r="C141" s="1223" t="n"/>
+      <c r="D141" s="1228" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="555" t="n"/>
+      <c r="B142" s="555" t="n"/>
+      <c r="C142" s="1223" t="n"/>
+      <c r="D142" s="1228" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="555" t="n"/>
+      <c r="B143" s="555" t="n"/>
+      <c r="C143" s="1223" t="n"/>
+      <c r="D143" s="1228" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="555" t="n"/>
+      <c r="B144" s="555" t="n"/>
+      <c r="C144" s="1223" t="n"/>
+      <c r="D144" s="1228" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="555" t="n"/>
+      <c r="B145" s="555" t="n"/>
+      <c r="C145" s="1223" t="n"/>
+      <c r="D145" s="1228" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="555" t="n"/>
+      <c r="B146" s="555" t="n"/>
+      <c r="C146" s="1223" t="n"/>
+      <c r="D146" s="1228" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="555" t="n"/>
+      <c r="B147" s="555" t="n"/>
+      <c r="C147" s="1223" t="n"/>
+      <c r="D147" s="1228" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="555" t="n"/>
+      <c r="B148" s="555" t="n"/>
+      <c r="C148" s="1223" t="n"/>
+      <c r="D148" s="1228" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="555" t="n"/>
+      <c r="B149" s="555" t="n"/>
+      <c r="C149" s="1223" t="n"/>
+      <c r="D149" s="1228" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="555" t="n"/>
+      <c r="B150" s="555" t="n"/>
+      <c r="C150" s="1223" t="n"/>
+      <c r="D150" s="1228" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="555" t="n"/>
+      <c r="B151" s="555" t="n"/>
+      <c r="C151" s="1223" t="n"/>
+      <c r="D151" s="1229" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="555" t="n"/>
+      <c r="B152" s="555" t="n"/>
+      <c r="C152" s="1223" t="n"/>
+      <c r="D152" s="1230" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="555" t="n"/>
+      <c r="B153" s="555" t="n"/>
+      <c r="C153" s="1223" t="n"/>
+      <c r="D153" s="1228" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="555" t="n"/>
+      <c r="B154" s="555" t="n"/>
+      <c r="C154" s="1223" t="n"/>
+      <c r="D154" s="1228" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="555" t="n"/>
+      <c r="B155" s="555" t="n"/>
+      <c r="C155" s="1223" t="n"/>
+      <c r="D155" s="1229" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="555" t="n"/>
+      <c r="B156" s="555" t="n"/>
+      <c r="C156" s="1223" t="n"/>
+      <c r="D156" s="1230" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="555" t="n"/>
+      <c r="B157" s="555" t="n"/>
+      <c r="C157" s="1223" t="n"/>
+      <c r="D157" s="1228" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="555" t="n"/>
+      <c r="B158" s="555" t="n"/>
+      <c r="C158" s="1223" t="n"/>
+      <c r="D158" s="1228" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="555" t="n"/>
+      <c r="B159" s="555" t="n"/>
+      <c r="C159" s="1223" t="n"/>
+      <c r="D159" s="1228" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="555" t="n"/>
+      <c r="B160" s="555" t="n"/>
+      <c r="C160" s="1223" t="n"/>
+      <c r="D160" s="1228" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="555" t="n"/>
+      <c r="B161" s="555" t="n"/>
+      <c r="C161" s="1223" t="n"/>
+      <c r="D161" s="1228" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="555" t="n"/>
+      <c r="B162" s="555" t="n"/>
+      <c r="C162" s="1223" t="n"/>
+      <c r="D162" s="1228" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="555" t="n"/>
+      <c r="B163" s="555" t="n"/>
+      <c r="C163" s="1223" t="n"/>
+      <c r="D163" s="1228" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="555" t="n"/>
+      <c r="B164" s="555" t="n"/>
+      <c r="C164" s="1223" t="n"/>
+      <c r="D164" s="1228" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="555" t="n"/>
+      <c r="B165" s="555" t="n"/>
+      <c r="C165" s="1223" t="n"/>
+      <c r="D165" s="1228" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="555" t="n"/>
+      <c r="B166" s="555" t="n"/>
+      <c r="C166" s="1223" t="n"/>
+      <c r="D166" s="1228" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="555" t="n"/>
+      <c r="B167" s="555" t="n"/>
+      <c r="C167" s="1223" t="n"/>
+      <c r="D167" s="1228" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="555" t="n"/>
+      <c r="B168" s="555" t="n"/>
+      <c r="C168" s="1223" t="n"/>
+      <c r="D168" s="1228" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="555" t="n"/>
+      <c r="B169" s="555" t="n"/>
+      <c r="C169" s="1223" t="n"/>
+      <c r="D169" s="1228" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="555" t="n"/>
+      <c r="B170" s="555" t="n"/>
+      <c r="C170" s="1223" t="n"/>
+      <c r="D170" s="1228" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="555" t="n"/>
+      <c r="B171" s="555" t="n"/>
+      <c r="C171" s="1223" t="n"/>
+      <c r="D171" s="1228" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="555" t="n"/>
+      <c r="B172" s="555" t="n"/>
+      <c r="C172" s="1223" t="n"/>
+      <c r="D172" s="1228" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="555" t="n"/>
+      <c r="B173" s="555" t="n"/>
+      <c r="C173" s="1223" t="n"/>
+      <c r="D173" s="1228" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="555" t="n"/>
+      <c r="B174" s="555" t="n"/>
+      <c r="C174" s="1223" t="n"/>
+      <c r="D174" s="1228" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="555" t="n"/>
+      <c r="B175" s="555" t="n"/>
+      <c r="C175" s="1223" t="n"/>
+      <c r="D175" s="1228" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="555" t="n"/>
+      <c r="B176" s="555" t="n"/>
+      <c r="C176" s="1223" t="n"/>
+      <c r="D176" s="1228" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="555" t="n"/>
+      <c r="B177" s="555" t="n"/>
+      <c r="C177" s="1223" t="n"/>
+      <c r="D177" s="1228" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="555" t="n"/>
+      <c r="B178" s="555" t="n"/>
+      <c r="C178" s="1223" t="n"/>
+      <c r="D178" s="1228" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="555" t="n"/>
+      <c r="B179" s="555" t="n"/>
+      <c r="C179" s="1223" t="n"/>
+      <c r="D179" s="1228" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="555" t="n"/>
+      <c r="B180" s="555" t="n"/>
+      <c r="C180" s="1223" t="n"/>
+      <c r="D180" s="1228" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="555" t="n"/>
+      <c r="B181" s="555" t="n"/>
+      <c r="C181" s="1223" t="n"/>
+      <c r="D181" s="1228" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="555" t="n"/>
+      <c r="B182" s="555" t="n"/>
+      <c r="C182" s="1223" t="n"/>
+      <c r="D182" s="1228" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="555" t="n"/>
+      <c r="B183" s="555" t="n"/>
+      <c r="C183" s="1223" t="n"/>
+      <c r="D183" s="1228" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="555" t="n"/>
+      <c r="B184" s="555" t="n"/>
+      <c r="C184" s="1223" t="n"/>
+      <c r="D184" s="1228" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="555" t="n"/>
+      <c r="B185" s="555" t="n"/>
+      <c r="C185" s="1223" t="n"/>
+      <c r="D185" s="1228" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="555" t="n"/>
+      <c r="B186" s="555" t="n"/>
+      <c r="C186" s="1223" t="n"/>
+      <c r="D186" s="1228" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="555" t="n"/>
+      <c r="B187" s="555" t="n"/>
+      <c r="C187" s="1223" t="n"/>
+      <c r="D187" s="1228" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="555" t="n"/>
+      <c r="B188" s="555" t="n"/>
+      <c r="C188" s="1223" t="n"/>
+      <c r="D188" s="1228" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="555" t="n"/>
+      <c r="B189" s="555" t="n"/>
+      <c r="C189" s="1223" t="n"/>
+      <c r="D189" s="1228" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="555" t="n"/>
+      <c r="B190" s="555" t="n"/>
+      <c r="C190" s="1223" t="n"/>
+      <c r="D190" s="1228" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="555" t="n"/>
+      <c r="B191" s="555" t="n"/>
+      <c r="C191" s="1223" t="n"/>
+      <c r="D191" s="1228" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="555" t="n"/>
+      <c r="B192" s="555" t="n"/>
+      <c r="C192" s="1223" t="n"/>
+      <c r="D192" s="1228" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="555" t="n"/>
+      <c r="B193" s="555" t="n"/>
+      <c r="C193" s="1223" t="n"/>
+      <c r="D193" s="1228" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="555" t="n"/>
+      <c r="B194" s="555" t="n"/>
+      <c r="C194" s="1223" t="n"/>
+      <c r="D194" s="1228" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="555" t="n"/>
+      <c r="B195" s="555" t="n"/>
+      <c r="C195" s="1223" t="n"/>
+      <c r="D195" s="1228" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="555" t="n"/>
+      <c r="B196" s="555" t="n"/>
+      <c r="C196" s="1223" t="n"/>
+      <c r="D196" s="1228" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="555" t="n"/>
+      <c r="B197" s="555" t="n"/>
+      <c r="C197" s="1223" t="n"/>
+      <c r="D197" s="1228" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="555" t="n"/>
+      <c r="B198" s="555" t="n"/>
+      <c r="C198" s="1223" t="n"/>
+      <c r="D198" s="1228" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="555" t="n"/>
+      <c r="B199" s="555" t="n"/>
+      <c r="C199" s="1223" t="n"/>
+      <c r="D199" s="1228" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="555" t="n"/>
+      <c r="B200" s="555" t="n"/>
+      <c r="C200" s="1223" t="n"/>
+      <c r="D200" s="1228" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="555" t="n"/>
+      <c r="B201" s="555" t="n"/>
+      <c r="C201" s="1223" t="n"/>
+      <c r="D201" s="1228" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="555" t="n"/>
+      <c r="B202" s="555" t="n"/>
+      <c r="C202" s="1223" t="n"/>
+      <c r="D202" s="1228" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="555" t="n"/>
+      <c r="B203" s="555" t="n"/>
+      <c r="C203" s="1223" t="n"/>
+      <c r="D203" s="1228" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="555" t="n"/>
+      <c r="B204" s="555" t="n"/>
+      <c r="C204" s="1223" t="n"/>
+      <c r="D204" s="1228" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="555" t="n"/>
+      <c r="B205" s="555" t="n"/>
+      <c r="C205" s="1223" t="n"/>
+      <c r="D205" s="1228" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="555" t="n"/>
+      <c r="B206" s="555" t="n"/>
+      <c r="C206" s="1223" t="n"/>
+      <c r="D206" s="1228" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="555" t="n"/>
+      <c r="B207" s="555" t="n"/>
+      <c r="C207" s="1223" t="n"/>
+      <c r="D207" s="1228" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="555" t="n"/>
+      <c r="B208" s="555" t="n"/>
+      <c r="C208" s="1223" t="n"/>
+      <c r="D208" s="1228" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="555" t="n"/>
+      <c r="B209" s="555" t="n"/>
+      <c r="C209" s="1223" t="n"/>
+      <c r="D209" s="1228" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="555" t="n"/>
+      <c r="B210" s="555" t="n"/>
+      <c r="C210" s="1223" t="n"/>
+      <c r="D210" s="1228" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="555" t="n"/>
+      <c r="B211" s="555" t="n"/>
+      <c r="C211" s="1223" t="n"/>
+      <c r="D211" s="1228" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="555" t="n"/>
+      <c r="B212" s="555" t="n"/>
+      <c r="C212" s="1223" t="n"/>
+      <c r="D212" s="1228" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="555" t="n"/>
+      <c r="B213" s="555" t="n"/>
+      <c r="C213" s="1223" t="n"/>
+      <c r="D213" s="1228" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="555" t="n"/>
+      <c r="B214" s="555" t="n"/>
+      <c r="C214" s="1223" t="n"/>
+      <c r="D214" s="1228" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="555" t="n"/>
+      <c r="B215" s="555" t="n"/>
+      <c r="C215" s="1223" t="n"/>
+      <c r="D215" s="1228" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="555" t="n"/>
+      <c r="B216" s="555" t="n"/>
+      <c r="C216" s="1223" t="n"/>
+      <c r="D216" s="1228" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="555" t="n"/>
+      <c r="B217" s="555" t="n"/>
+      <c r="C217" s="1223" t="n"/>
+      <c r="D217" s="1228" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="555" t="n"/>
+      <c r="B218" s="555" t="n"/>
+      <c r="C218" s="1223" t="n"/>
+      <c r="D218" s="1228" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="555" t="n"/>
+      <c r="B219" s="555" t="n"/>
+      <c r="C219" s="1223" t="n"/>
+      <c r="D219" s="1228" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="555" t="n"/>
+      <c r="B220" s="555" t="n"/>
+      <c r="C220" s="1223" t="n"/>
+      <c r="D220" s="1228" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="555" t="n"/>
+      <c r="B221" s="555" t="n"/>
+      <c r="C221" s="1223" t="n"/>
+      <c r="D221" s="1228" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="555" t="n"/>
+      <c r="B222" s="555" t="n"/>
+      <c r="C222" s="1223" t="n"/>
+      <c r="D222" s="1228" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="555" t="n"/>
+      <c r="B223" s="555" t="n"/>
+      <c r="C223" s="1223" t="n"/>
+      <c r="D223" s="1228" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="555" t="n"/>
+      <c r="B224" s="555" t="n"/>
+      <c r="C224" s="1223" t="n"/>
+      <c r="D224" s="1228" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="555" t="n"/>
+      <c r="B225" s="555" t="n"/>
+      <c r="C225" s="1223" t="n"/>
+      <c r="D225" s="1228" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="555" t="n"/>
+      <c r="B226" s="555" t="n"/>
+      <c r="C226" s="1223" t="n"/>
+      <c r="D226" s="1228" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="555" t="n"/>
+      <c r="B227" s="555" t="n"/>
+      <c r="C227" s="1223" t="n"/>
+      <c r="D227" s="1228" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="555" t="n"/>
+      <c r="B228" s="555" t="n"/>
+      <c r="C228" s="1223" t="n"/>
+      <c r="D228" s="1228" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="555" t="n"/>
+      <c r="B229" s="555" t="n"/>
+      <c r="C229" s="1223" t="n"/>
+      <c r="D229" s="1228" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="555" t="n"/>
+      <c r="B230" s="555" t="n"/>
+      <c r="C230" s="1223" t="n"/>
+      <c r="D230" s="1228" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="555" t="n"/>
+      <c r="B231" s="555" t="n"/>
+      <c r="C231" s="1223" t="n"/>
+      <c r="D231" s="1228" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="555" t="n"/>
+      <c r="B232" s="555" t="n"/>
+      <c r="C232" s="1223" t="n"/>
+      <c r="D232" s="1228" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="555" t="n"/>
+      <c r="B233" s="555" t="n"/>
+      <c r="C233" s="1223" t="n"/>
+      <c r="D233" s="1228" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="555" t="n"/>
+      <c r="B234" s="555" t="n"/>
+      <c r="C234" s="1223" t="n"/>
+      <c r="D234" s="1228" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="555" t="n"/>
+      <c r="B235" s="555" t="n"/>
+      <c r="C235" s="1223" t="n"/>
+      <c r="D235" s="1228" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="555" t="n"/>
+      <c r="B236" s="555" t="n"/>
+      <c r="C236" s="1223" t="n"/>
+      <c r="D236" s="1228" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="555" t="n"/>
+      <c r="B237" s="555" t="n"/>
+      <c r="C237" s="1223" t="n"/>
+      <c r="D237" s="1228" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="555" t="n"/>
+      <c r="B238" s="555" t="n"/>
+      <c r="C238" s="1223" t="n"/>
+      <c r="D238" s="1228" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="555" t="n"/>
+      <c r="B239" s="555" t="n"/>
+      <c r="C239" s="1223" t="n"/>
+      <c r="D239" s="1228" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="555" t="n"/>
+      <c r="B240" s="555" t="n"/>
+      <c r="C240" s="1223" t="n"/>
+      <c r="D240" s="1228" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="555" t="n"/>
+      <c r="B241" s="555" t="n"/>
+      <c r="C241" s="1223" t="n"/>
+      <c r="D241" s="1228" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="555" t="n"/>
+      <c r="B242" s="555" t="n"/>
+      <c r="C242" s="1223" t="n"/>
+      <c r="D242" s="1228" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="555" t="n"/>
+      <c r="B243" s="555" t="n"/>
+      <c r="C243" s="1223" t="n"/>
+      <c r="D243" s="1228" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="555" t="n"/>
+      <c r="B244" s="555" t="n"/>
+      <c r="C244" s="1223" t="n"/>
+      <c r="D244" s="1228" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="555" t="n"/>
+      <c r="B245" s="555" t="n"/>
+      <c r="C245" s="1223" t="n"/>
+      <c r="D245" s="1228" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="555" t="n"/>
+      <c r="B246" s="555" t="n"/>
+      <c r="C246" s="1223" t="n"/>
+      <c r="D246" s="1228" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="555" t="n"/>
+      <c r="B247" s="555" t="n"/>
+      <c r="C247" s="1223" t="n"/>
+      <c r="D247" s="1228" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="555" t="n"/>
+      <c r="B248" s="555" t="n"/>
+      <c r="C248" s="1223" t="n"/>
+      <c r="D248" s="1228" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="555" t="n"/>
+      <c r="B249" s="555" t="n"/>
+      <c r="C249" s="1223" t="n"/>
+      <c r="D249" s="1228" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="555" t="n"/>
+      <c r="B250" s="555" t="n"/>
+      <c r="C250" s="1223" t="n"/>
+      <c r="D250" s="1228" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="555" t="n"/>
+      <c r="B251" s="555" t="n"/>
+      <c r="C251" s="1223" t="n"/>
+      <c r="D251" s="1228" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="555" t="n"/>
+      <c r="B252" s="555" t="n"/>
+      <c r="C252" s="1223" t="n"/>
+      <c r="D252" s="1228" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="555" t="n"/>
+      <c r="B253" s="555" t="n"/>
+      <c r="C253" s="1223" t="n"/>
+      <c r="D253" s="1228" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="555" t="n"/>
+      <c r="B254" s="555" t="n"/>
+      <c r="C254" s="1223" t="n"/>
+      <c r="D254" s="1228" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="555" t="n"/>
+      <c r="B255" s="555" t="n"/>
+      <c r="C255" s="1223" t="n"/>
+      <c r="D255" s="1228" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="555" t="n"/>
+      <c r="B256" s="555" t="n"/>
+      <c r="C256" s="1223" t="n"/>
+      <c r="D256" s="1228" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="555" t="n"/>
+      <c r="B257" s="555" t="n"/>
+      <c r="C257" s="1223" t="n"/>
+      <c r="D257" s="1228" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="555" t="n"/>
+      <c r="B258" s="555" t="n"/>
+      <c r="C258" s="1223" t="n"/>
+      <c r="D258" s="1228" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="555" t="n"/>
+      <c r="B259" s="555" t="n"/>
+      <c r="C259" s="1223" t="n"/>
+      <c r="D259" s="1228" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="555" t="n"/>
+      <c r="B260" s="555" t="n"/>
+      <c r="C260" s="1223" t="n"/>
+      <c r="D260" s="1228" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="555" t="n"/>
+      <c r="B261" s="555" t="n"/>
+      <c r="C261" s="1223" t="n"/>
+      <c r="D261" s="1228" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="555" t="n"/>
+      <c r="B262" s="555" t="n"/>
+      <c r="C262" s="1223" t="n"/>
+      <c r="D262" s="1228" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="555" t="n"/>
+      <c r="B263" s="555" t="n"/>
+      <c r="C263" s="1223" t="n"/>
+      <c r="D263" s="1228" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="555" t="n"/>
+      <c r="B264" s="555" t="n"/>
+      <c r="C264" s="1223" t="n"/>
+      <c r="D264" s="1228" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="555" t="n"/>
+      <c r="B265" s="555" t="n"/>
+      <c r="C265" s="1223" t="n"/>
+      <c r="D265" s="1228" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="555" t="n"/>
+      <c r="B266" s="555" t="n"/>
+      <c r="C266" s="1223" t="n"/>
+      <c r="D266" s="1228" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="555" t="n"/>
+      <c r="B267" s="555" t="n"/>
+      <c r="C267" s="1223" t="n"/>
+      <c r="D267" s="1228" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="555" t="n"/>
+      <c r="B268" s="555" t="n"/>
+      <c r="C268" s="1223" t="n"/>
+      <c r="D268" s="1228" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="555" t="n"/>
+      <c r="B269" s="555" t="n"/>
+      <c r="C269" s="1223" t="n"/>
+      <c r="D269" s="1228" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="555" t="n"/>
+      <c r="B270" s="555" t="n"/>
+      <c r="C270" s="1223" t="n"/>
+      <c r="D270" s="1228" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="555" t="n"/>
+      <c r="B271" s="555" t="n"/>
+      <c r="C271" s="1223" t="n"/>
+      <c r="D271" s="1228" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="555" t="n"/>
+      <c r="B272" s="555" t="n"/>
+      <c r="C272" s="1223" t="n"/>
+      <c r="D272" s="1228" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="555" t="n"/>
+      <c r="B273" s="555" t="n"/>
+      <c r="C273" s="1223" t="n"/>
+      <c r="D273" s="1228" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="555" t="n"/>
+      <c r="B274" s="555" t="n"/>
+      <c r="C274" s="1223" t="n"/>
+      <c r="D274" s="1228" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="555" t="n"/>
+      <c r="B275" s="555" t="n"/>
+      <c r="C275" s="1223" t="n"/>
+      <c r="D275" s="1228" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="555" t="n"/>
+      <c r="B276" s="555" t="n"/>
+      <c r="C276" s="1223" t="n"/>
+      <c r="D276" s="1228" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="555" t="n"/>
+      <c r="B277" s="555" t="n"/>
+      <c r="C277" s="1223" t="n"/>
+      <c r="D277" s="1228" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="555" t="n"/>
+      <c r="B278" s="555" t="n"/>
+      <c r="C278" s="1223" t="n"/>
+      <c r="D278" s="1228" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="555" t="n"/>
+      <c r="B279" s="555" t="n"/>
+      <c r="C279" s="1223" t="n"/>
+      <c r="D279" s="1228" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="555" t="n"/>
+      <c r="B280" s="555" t="n"/>
+      <c r="C280" s="1223" t="n"/>
+      <c r="D280" s="1228" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="555" t="n"/>
+      <c r="B281" s="555" t="n"/>
+      <c r="C281" s="1223" t="n"/>
+      <c r="D281" s="1228" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="555" t="n"/>
+      <c r="B282" s="555" t="n"/>
+      <c r="C282" s="1223" t="n"/>
+      <c r="D282" s="1228" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="555" t="n"/>
+      <c r="B283" s="555" t="n"/>
+      <c r="C283" s="1223" t="n"/>
+      <c r="D283" s="1228" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="555" t="n"/>
+      <c r="B284" s="555" t="n"/>
+      <c r="C284" s="1223" t="n"/>
+      <c r="D284" s="1228" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="555" t="n"/>
+      <c r="B285" s="555" t="n"/>
+      <c r="C285" s="1223" t="n"/>
+      <c r="D285" s="1228" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="555" t="n"/>
+      <c r="B286" s="555" t="n"/>
+      <c r="C286" s="1223" t="n"/>
+      <c r="D286" s="1228" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="555" t="n"/>
+      <c r="B287" s="555" t="n"/>
+      <c r="C287" s="1223" t="n"/>
+      <c r="D287" s="1228" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="555" t="n"/>
+      <c r="B288" s="555" t="n"/>
+      <c r="C288" s="1223" t="n"/>
+      <c r="D288" s="1228" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="555" t="n"/>
+      <c r="B289" s="555" t="n"/>
+      <c r="C289" s="1223" t="n"/>
+      <c r="D289" s="1228" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="555" t="n"/>
+      <c r="B290" s="555" t="n"/>
+      <c r="C290" s="1223" t="n"/>
+      <c r="D290" s="1228" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="555" t="n"/>
+      <c r="B291" s="555" t="n"/>
+      <c r="C291" s="1223" t="n"/>
+      <c r="D291" s="1228" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="555" t="n"/>
+      <c r="B292" s="555" t="n"/>
+      <c r="C292" s="1223" t="n"/>
+      <c r="D292" s="1228" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="555" t="n"/>
+      <c r="B293" s="555" t="n"/>
+      <c r="C293" s="1223" t="n"/>
+      <c r="D293" s="1228" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="555" t="n"/>
+      <c r="B294" s="555" t="n"/>
+      <c r="C294" s="1223" t="n"/>
+      <c r="D294" s="1228" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="555" t="n"/>
+      <c r="B295" s="555" t="n"/>
+      <c r="C295" s="1223" t="n"/>
+      <c r="D295" s="1228" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="555" t="n"/>
+      <c r="B296" s="555" t="n"/>
+      <c r="C296" s="1223" t="n"/>
+      <c r="D296" s="1228" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="555" t="n"/>
+      <c r="B297" s="555" t="n"/>
+      <c r="C297" s="1223" t="n"/>
+      <c r="D297" s="1228" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="555" t="n"/>
+      <c r="B298" s="555" t="n"/>
+      <c r="C298" s="1223" t="n"/>
+      <c r="D298" s="1228" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="555" t="n"/>
+      <c r="B299" s="555" t="n"/>
+      <c r="C299" s="1223" t="n"/>
+      <c r="D299" s="1228" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="555" t="n"/>
+      <c r="B300" s="555" t="n"/>
+      <c r="C300" s="1223" t="n"/>
+      <c r="D300" s="1228" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="555" t="n"/>
+      <c r="B301" s="555" t="n"/>
+      <c r="C301" s="1223" t="n"/>
+      <c r="D301" s="1228" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="555" t="n"/>
+      <c r="B302" s="555" t="n"/>
+      <c r="C302" s="1223" t="n"/>
+      <c r="D302" s="1228" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="555" t="n"/>
+      <c r="B303" s="555" t="n"/>
+      <c r="C303" s="1223" t="n"/>
+      <c r="D303" s="1228" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="555" t="n"/>
+      <c r="B304" s="555" t="n"/>
+      <c r="C304" s="1223" t="n"/>
+      <c r="D304" s="1228" t="n"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="555" t="n"/>
+      <c r="B305" s="555" t="n"/>
+      <c r="C305" s="1223" t="n"/>
+      <c r="D305" s="1228" t="n"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="555" t="n"/>
+      <c r="B306" s="555" t="n"/>
+      <c r="C306" s="1223" t="n"/>
+      <c r="D306" s="1228" t="n"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="555" t="n"/>
+      <c r="B307" s="555" t="n"/>
+      <c r="C307" s="1223" t="n"/>
+      <c r="D307" s="1228" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="555" t="n"/>
+      <c r="B308" s="555" t="n"/>
+      <c r="C308" s="1223" t="n"/>
+      <c r="D308" s="1228" t="n"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="555" t="n"/>
+      <c r="B309" s="555" t="n"/>
+      <c r="C309" s="1223" t="n"/>
+      <c r="D309" s="1228" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="555" t="n"/>
+      <c r="B310" s="555" t="n"/>
+      <c r="C310" s="1223" t="n"/>
+      <c r="D310" s="1228" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="555" t="n"/>
+      <c r="B311" s="555" t="n"/>
+      <c r="C311" s="1223" t="n"/>
+      <c r="D311" s="1228" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="555" t="n"/>
+      <c r="B312" s="555" t="n"/>
+      <c r="C312" s="1223" t="n"/>
+      <c r="D312" s="1228" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="555" t="n"/>
+      <c r="B313" s="555" t="n"/>
+      <c r="C313" s="1223" t="n"/>
+      <c r="D313" s="1228" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="555" t="n"/>
+      <c r="B314" s="555" t="n"/>
+      <c r="C314" s="1223" t="n"/>
+      <c r="D314" s="1228" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="555" t="n"/>
+      <c r="B315" s="555" t="n"/>
+      <c r="C315" s="1223" t="n"/>
+      <c r="D315" s="1228" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="555" t="n"/>
+      <c r="B316" s="555" t="n"/>
+      <c r="C316" s="1223" t="n"/>
+      <c r="D316" s="1228" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="555" t="n"/>
+      <c r="B317" s="555" t="n"/>
+      <c r="C317" s="1223" t="n"/>
+      <c r="D317" s="1228" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="555" t="n"/>
+      <c r="B318" s="555" t="n"/>
+      <c r="C318" s="1223" t="n"/>
+      <c r="D318" s="1228" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="555" t="n"/>
+      <c r="B319" s="555" t="n"/>
+      <c r="C319" s="1223" t="n"/>
+      <c r="D319" s="1228" t="n"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="555" t="n"/>
+      <c r="B320" s="555" t="n"/>
+      <c r="C320" s="1223" t="n"/>
+      <c r="D320" s="1228" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="555" t="n"/>
+      <c r="B321" s="555" t="n"/>
+      <c r="C321" s="1223" t="n"/>
+      <c r="D321" s="1228" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="555" t="n"/>
+      <c r="B322" s="555" t="n"/>
+      <c r="C322" s="1223" t="n"/>
+      <c r="D322" s="1228" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="555" t="n"/>
+      <c r="B323" s="555" t="n"/>
+      <c r="C323" s="1223" t="n"/>
+      <c r="D323" s="1228" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="555" t="n"/>
+      <c r="B324" s="555" t="n"/>
+      <c r="C324" s="1223" t="n"/>
+      <c r="D324" s="1228" t="n"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="555" t="n"/>
+      <c r="B325" s="555" t="n"/>
+      <c r="C325" s="1223" t="n"/>
+      <c r="D325" s="1228" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="555" t="n"/>
+      <c r="B326" s="555" t="n"/>
+      <c r="C326" s="1223" t="n"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="555" t="n"/>
+      <c r="B327" s="555" t="n"/>
+      <c r="C327" s="1223" t="n"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="555" t="n"/>
+      <c r="B328" s="555" t="n"/>
+      <c r="C328" s="1223" t="n"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="555" t="n"/>
+      <c r="B329" s="555" t="n"/>
+      <c r="C329" s="1223" t="n"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="555" t="n"/>
+      <c r="B330" s="555" t="n"/>
+      <c r="C330" s="1223" t="n"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="555" t="n"/>
+      <c r="B331" s="555" t="n"/>
+      <c r="C331" s="1223" t="n"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="555" t="n"/>
+      <c r="B332" s="555" t="n"/>
+      <c r="C332" s="1223" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="555" t="n"/>
+      <c r="B333" s="555" t="n"/>
+      <c r="C333" s="1223" t="n"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="555" t="n"/>
+      <c r="B334" s="555" t="n"/>
+      <c r="C334" s="1223" t="n"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="555" t="n"/>
+      <c r="B335" s="555" t="n"/>
+      <c r="C335" s="1223" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="0" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>